<commit_message>
main_mmixte (on ne choisit pas les PM )
</commit_message>
<xml_diff>
--- a/data/raw/FINAL_Defi_Access_Garches_22_05_2026_nettoye╠ü.xlsx
+++ b/data/raw/FINAL_Defi_Access_Garches_22_05_2026_nettoye╠ü.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EPF\STAGE ACCESS\Code\Prototype_Appli_DefisAccess\data\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/93c607bc84408f6b/Bureau/defi_access_aloïs/Prototype_Appli_DefisAccess/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD06BD7-6A1E-458B-9234-40B763A485CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{0AD06BD7-6A1E-458B-9234-40B763A485CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1EB685F-052C-4758-8AB8-DBC1AB126447}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="13248" windowHeight="6936" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -438,7 +438,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -454,6 +454,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -485,7 +497,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -507,6 +519,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1688,7 +1706,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="71" style="1" customWidth="1"/>
-    <col min="2" max="2" width="33.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.44140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" style="1" customWidth="1"/>
@@ -2650,7 +2668,7 @@
       </c>
       <c r="D53" s="5"/>
       <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
+      <c r="F53" s="9"/>
       <c r="G53" s="6"/>
     </row>
     <row r="54" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2686,7 +2704,7 @@
         <v>1</v>
       </c>
       <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
+      <c r="F55" s="8"/>
       <c r="G55" s="6"/>
     </row>
     <row r="56" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2701,7 +2719,7 @@
       </c>
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
+      <c r="F56" s="9"/>
       <c r="G56" s="6"/>
     </row>
     <row r="57" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2735,7 +2753,7 @@
         <v>0</v>
       </c>
       <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
+      <c r="F58" s="8"/>
       <c r="G58" s="3" t="s">
         <v>24</v>
       </c>
@@ -2848,7 +2866,7 @@
       <c r="E65" s="5">
         <v>0</v>
       </c>
-      <c r="F65" s="5"/>
+      <c r="F65" s="9"/>
       <c r="G65" s="3" t="s">
         <v>83</v>
       </c>
@@ -2869,7 +2887,7 @@
       <c r="E66" s="5">
         <v>0</v>
       </c>
-      <c r="F66" s="5"/>
+      <c r="F66" s="9"/>
       <c r="G66" s="3" t="s">
         <v>85</v>
       </c>
@@ -2924,7 +2942,7 @@
         <v>0.5</v>
       </c>
       <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
+      <c r="F69" s="8"/>
       <c r="G69" s="6"/>
     </row>
     <row r="70" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2977,7 +2995,7 @@
         <v>0.5</v>
       </c>
       <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
+      <c r="F72" s="8"/>
       <c r="G72" s="6"/>
     </row>
     <row r="73" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3009,7 +3027,7 @@
       </c>
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
-      <c r="F74" s="5"/>
+      <c r="F74" s="8"/>
       <c r="G74" s="6"/>
     </row>
     <row r="75" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3045,7 +3063,7 @@
         <v>0.5</v>
       </c>
       <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
+      <c r="F76" s="8"/>
       <c r="G76" s="6"/>
     </row>
     <row r="77" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3081,7 +3099,7 @@
         <v>1</v>
       </c>
       <c r="E78" s="5"/>
-      <c r="F78" s="5"/>
+      <c r="F78" s="8"/>
       <c r="G78" s="6"/>
     </row>
     <row r="79" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3098,7 +3116,7 @@
         <v>1</v>
       </c>
       <c r="E79" s="5"/>
-      <c r="F79" s="5"/>
+      <c r="F79" s="8"/>
       <c r="G79" s="3" t="s">
         <v>102</v>
       </c>
@@ -3172,7 +3190,7 @@
         <v>1</v>
       </c>
       <c r="E83" s="5"/>
-      <c r="F83" s="5"/>
+      <c r="F83" s="8"/>
       <c r="G83" s="3" t="s">
         <v>105</v>
       </c>
@@ -3191,7 +3209,7 @@
         <v>0</v>
       </c>
       <c r="E84" s="5"/>
-      <c r="F84" s="5"/>
+      <c r="F84" s="8"/>
       <c r="G84" s="3" t="s">
         <v>102</v>
       </c>
@@ -3227,7 +3245,7 @@
         <v>0</v>
       </c>
       <c r="E86" s="5"/>
-      <c r="F86" s="5"/>
+      <c r="F86" s="8"/>
       <c r="G86" s="3" t="s">
         <v>102</v>
       </c>
@@ -3282,7 +3300,7 @@
         <v>1</v>
       </c>
       <c r="E89" s="5"/>
-      <c r="F89" s="5"/>
+      <c r="F89" s="8"/>
       <c r="G89" s="3" t="s">
         <v>112</v>
       </c>
@@ -3341,7 +3359,7 @@
       <c r="E92" s="5">
         <v>1</v>
       </c>
-      <c r="F92" s="5"/>
+      <c r="F92" s="8"/>
       <c r="G92" s="6"/>
     </row>
     <row r="93" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3400,7 +3418,7 @@
       <c r="E95" s="5">
         <v>1</v>
       </c>
-      <c r="F95" s="5"/>
+      <c r="F95" s="8"/>
       <c r="G95" s="6"/>
     </row>
     <row r="96" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3434,7 +3452,7 @@
         <v>1</v>
       </c>
       <c r="E97" s="5"/>
-      <c r="F97" s="5"/>
+      <c r="F97" s="8"/>
       <c r="G97" s="3" t="s">
         <v>24</v>
       </c>
@@ -3453,7 +3471,7 @@
         <v>0</v>
       </c>
       <c r="E98" s="5"/>
-      <c r="F98" s="5"/>
+      <c r="F98" s="8"/>
       <c r="G98" s="6"/>
     </row>
     <row r="99" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3506,7 +3524,7 @@
         <v>1</v>
       </c>
       <c r="E101" s="5"/>
-      <c r="F101" s="5"/>
+      <c r="F101" s="9"/>
       <c r="G101" s="3" t="s">
         <v>24</v>
       </c>
@@ -3548,7 +3566,7 @@
       <c r="E103" s="5">
         <v>1</v>
       </c>
-      <c r="F103" s="5"/>
+      <c r="F103" s="8"/>
       <c r="G103" s="3" t="s">
         <v>128</v>
       </c>
@@ -3588,7 +3606,7 @@
       <c r="E105" s="5">
         <v>1</v>
       </c>
-      <c r="F105" s="5"/>
+      <c r="F105" s="10"/>
       <c r="G105" s="6"/>
     </row>
   </sheetData>

</xml_diff>